<commit_message>
Actualiza documentos y sistema exclusivamente dentro de Fase 2
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencia Proyecto/Evidencias Documentacion/06_Carta_Gantt_PMP_Suite_V2.0.xlsx
+++ b/Fase 2/Evidencia Proyecto/Evidencias Documentacion/06_Carta_Gantt_PMP_Suite_V2.0.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -589,8 +589,10 @@
     </row>
     <row r="2" ht="33" customHeight="1">
       <c r="A2" s="3"/>
-      <c r="B2" s="4" t="str">
-        <v>Carta Gantt PMP Suite</v>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Carta Gantt PMP Suite V2.0</t>
+        </is>
       </c>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
@@ -618,8 +620,10 @@
     </row>
     <row r="3" ht="25" customHeight="1">
       <c r="A3" s="3"/>
-      <c r="B3" s="5" t="str">
-        <v>Plan de trabajo desde la definición hasta el cierre. Semanas relativas 1 a 18.</v>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Planificación basal en cascada. Semanas relativas 1 a 18; sin fechas calendario ni avance ejecutado.</t>
+        </is>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5"/>
@@ -1905,8 +1909,10 @@
     </row>
     <row r="25" ht="25" customHeight="1">
       <c r="A25" s="3"/>
-      <c r="B25" s="6" t="str">
-        <v>Fuente: plan de trabajo proporcionado por el usuario.</v>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Referencia: Acta de Constitución V2.0, sección 2. Los hitos son puntos de control; no acreditan aprobaciones.</t>
+        </is>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>

</xml_diff>